<commit_message>
Updated: Retry Scenario Position Added
</commit_message>
<xml_diff>
--- a/Config/Client_Config.xlsx
+++ b/Config/Client_Config.xlsx
@@ -28,7 +28,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="36" uniqueCount="31">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="34" uniqueCount="29">
   <si>
     <t>Branch Name</t>
   </si>
@@ -81,27 +81,15 @@
     <t>SenderEmail</t>
   </si>
   <si>
-    <t>testquadan@gmail.com</t>
-  </si>
-  <si>
     <t>EmailPassword</t>
   </si>
   <si>
-    <t>ldpa zvpf wqkm tukc</t>
-  </si>
-  <si>
     <t>StatusFolderId  </t>
   </si>
   <si>
     <t>RootFolderId</t>
   </si>
   <si>
-    <t>StatusFileName</t>
-  </si>
-  <si>
-    <t>StatusTracker.xlsx</t>
-  </si>
-  <si>
     <t>1nBXAMP28x_bG5B_yFbg2vK_9D2ckjaKT</t>
   </si>
   <si>
@@ -121,6 +109,12 @@
   </si>
   <si>
     <t>TMCV-Ser-S-CHN-1001860-Madhavaram-DSvCM</t>
+  </si>
+  <si>
+    <t>cor.rpa.srvclaims@pmmil.com</t>
+  </si>
+  <si>
+    <t>udzn ybdc jaif akvx</t>
   </si>
 </sst>
 </file>
@@ -629,16 +623,16 @@
     </row>
     <row r="3" spans="1:5" ht="15">
       <c r="A3" s="11" t="s">
-        <v>26</v>
+        <v>22</v>
       </c>
       <c r="B3" s="14" t="s">
-        <v>27</v>
+        <v>23</v>
       </c>
       <c r="C3" s="10" t="s">
         <v>6</v>
       </c>
       <c r="D3" s="12" t="s">
-        <v>28</v>
+        <v>24</v>
       </c>
       <c r="E3" s="13" t="s">
         <v>5</v>
@@ -646,16 +640,16 @@
     </row>
     <row r="4" spans="1:5" ht="15">
       <c r="A4" s="11" t="s">
-        <v>29</v>
+        <v>25</v>
       </c>
       <c r="B4" s="14" t="s">
-        <v>27</v>
+        <v>23</v>
       </c>
       <c r="C4" s="10" t="s">
         <v>6</v>
       </c>
       <c r="D4" s="12" t="s">
-        <v>30</v>
+        <v>26</v>
       </c>
       <c r="E4" s="13" t="s">
         <v>5</v>
@@ -675,7 +669,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:B8"/>
+  <dimension ref="A1:B7"/>
   <sheetFormatPr defaultRowHeight="14.25"/>
   <cols>
     <col min="1" max="1" width="19.125" customWidth="1"/>
@@ -710,49 +704,64 @@
       <c r="A4" t="s">
         <v>16</v>
       </c>
-      <c r="B4" t="s">
-        <v>17</v>
+      <c r="B4" s="4" t="s">
+        <v>27</v>
       </c>
     </row>
     <row r="5" spans="1:2">
       <c r="A5" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="B5" t="s">
-        <v>19</v>
+        <v>28</v>
       </c>
     </row>
     <row r="6" spans="1:2">
       <c r="A6" t="s">
-        <v>20</v>
+        <v>18</v>
       </c>
       <c r="B6" t="s">
-        <v>25</v>
+        <v>21</v>
       </c>
     </row>
     <row r="7" spans="1:2">
       <c r="A7" t="s">
-        <v>21</v>
+        <v>19</v>
       </c>
       <c r="B7" t="s">
-        <v>24</v>
-      </c>
-    </row>
-    <row r="8" spans="1:2">
-      <c r="A8" t="s">
-        <v>22</v>
-      </c>
-      <c r="B8" t="s">
-        <v>23</v>
+        <v>20</v>
       </c>
     </row>
   </sheetData>
+  <hyperlinks>
+    <hyperlink ref="B4" r:id="rId1"/>
+  </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup orientation="portrait" r:id="rId1"/>
+  <pageSetup orientation="portrait" r:id="rId2"/>
 </worksheet>
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement>
+    <TaxCatchAll xmlns="399697c3-5931-482a-bf60-528e1410a718" xsi:nil="true"/>
+    <lcf76f155ced4ddcb4097134ff3c332f xmlns="69774094-9380-4fae-b934-13dda1a7dd00">
+      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    </lcf76f155ced4ddcb4097134ff3c332f>
+  </documentManagement>
+</p:properties>
+</file>
+
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
+</file>
+
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x01010044376E494BD8C84F84CDAE7F49671CB7" ma:contentTypeVersion="18" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="976d064ff5353b1784c9cc50294987ed">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="69774094-9380-4fae-b934-13dda1a7dd00" xmlns:ns3="399697c3-5931-482a-bf60-528e1410a718" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="6d25ac32989da96868f130ee3b29a1a8" ns2:_="" ns3:_="">
     <xsd:import namespace="69774094-9380-4fae-b934-13dda1a7dd00"/>
@@ -1007,27 +1016,26 @@
 </ct:contentTypeSchema>
 </file>
 
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
+<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{1EADD28A-BF2C-45E6-83DF-53D59D707908}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="399697c3-5931-482a-bf60-528e1410a718"/>
+    <ds:schemaRef ds:uri="69774094-9380-4fae-b934-13dda1a7dd00"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
 
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement>
-    <TaxCatchAll xmlns="399697c3-5931-482a-bf60-528e1410a718" xsi:nil="true"/>
-    <lcf76f155ced4ddcb4097134ff3c332f xmlns="69774094-9380-4fae-b934-13dda1a7dd00">
-      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    </lcf76f155ced4ddcb4097134ff3c332f>
-  </documentManagement>
-</p:properties>
+<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{065CC945-652E-4DFC-A1A9-9FF2FC932111}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
 
-<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{1860C180-34A5-4519-8E01-EE45D69AD4EA}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
@@ -1044,23 +1052,4 @@
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/internal/obd"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{065CC945-652E-4DFC-A1A9-9FF2FC932111}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{1EADD28A-BF2C-45E6-83DF-53D59D707908}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <ds:schemaRef ds:uri="399697c3-5931-482a-bf60-528e1410a718"/>
-    <ds:schemaRef ds:uri="69774094-9380-4fae-b934-13dda1a7dd00"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
 </file>
</xml_diff>

<commit_message>
Updated: Remove Files Keyword from RDP
</commit_message>
<xml_diff>
--- a/Config/Client_Config.xlsx
+++ b/Config/Client_Config.xlsx
@@ -12,11 +12,11 @@
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720"/>
   </bookViews>
   <sheets>
-    <sheet name="Sheet1" sheetId="4" r:id="rId1"/>
-    <sheet name="Sheet2" sheetId="5" r:id="rId2"/>
+    <sheet name="Login_Credentials" sheetId="4" r:id="rId1"/>
+    <sheet name="Other_Credentials" sheetId="5" r:id="rId2"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">Sheet1!$A$1:$E$4</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">Login_Credentials!$A$1:$E$4</definedName>
   </definedNames>
   <calcPr calcId="162913"/>
   <extLst>
@@ -28,7 +28,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="34" uniqueCount="30">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="38" uniqueCount="34">
   <si>
     <t>Branch Name</t>
   </si>
@@ -118,6 +118,18 @@
   </si>
   <si>
     <t>TMCV-Ser-S-TN1-1001860-Kattupakka-DSvCM</t>
+  </si>
+  <si>
+    <t>RecipientTo</t>
+  </si>
+  <si>
+    <t>vishnu.s@quadance.com;benly.polly@quadance.com</t>
+  </si>
+  <si>
+    <t>RecipientCc</t>
+  </si>
+  <si>
+    <t>vishnu.s@quadance.com</t>
   </si>
 </sst>
 </file>
@@ -669,11 +681,11 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:B7"/>
+  <dimension ref="A1:B9"/>
   <sheetFormatPr defaultRowHeight="14.25"/>
   <cols>
     <col min="1" max="1" width="19.125" customWidth="1"/>
-    <col min="2" max="2" width="36.375" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="45.5" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:2" ht="15">
@@ -732,16 +744,54 @@
         <v>16</v>
       </c>
     </row>
+    <row r="8" spans="1:2">
+      <c r="A8" s="12" t="s">
+        <v>30</v>
+      </c>
+      <c r="B8" s="4" t="s">
+        <v>31</v>
+      </c>
+    </row>
+    <row r="9" spans="1:2">
+      <c r="A9" s="12" t="s">
+        <v>32</v>
+      </c>
+      <c r="B9" s="4" t="s">
+        <v>33</v>
+      </c>
+    </row>
   </sheetData>
   <hyperlinks>
     <hyperlink ref="B4" r:id="rId1"/>
+    <hyperlink ref="B8" r:id="rId2"/>
+    <hyperlink ref="B9" r:id="rId3"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup orientation="portrait" r:id="rId2"/>
+  <pageSetup orientation="portrait" r:id="rId4"/>
 </worksheet>
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
+</file>
+
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement>
+    <TaxCatchAll xmlns="399697c3-5931-482a-bf60-528e1410a718" xsi:nil="true"/>
+    <lcf76f155ced4ddcb4097134ff3c332f xmlns="69774094-9380-4fae-b934-13dda1a7dd00">
+      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    </lcf76f155ced4ddcb4097134ff3c332f>
+  </documentManagement>
+</p:properties>
+</file>
+
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x01010044376E494BD8C84F84CDAE7F49671CB7" ma:contentTypeVersion="18" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="976d064ff5353b1784c9cc50294987ed">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="69774094-9380-4fae-b934-13dda1a7dd00" xmlns:ns3="399697c3-5931-482a-bf60-528e1410a718" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="6d25ac32989da96868f130ee3b29a1a8" ns2:_="" ns3:_="">
     <xsd:import namespace="69774094-9380-4fae-b934-13dda1a7dd00"/>
@@ -996,27 +1046,26 @@
 </ct:contentTypeSchema>
 </file>
 
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
+<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{065CC945-652E-4DFC-A1A9-9FF2FC932111}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
 
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement>
-    <TaxCatchAll xmlns="399697c3-5931-482a-bf60-528e1410a718" xsi:nil="true"/>
-    <lcf76f155ced4ddcb4097134ff3c332f xmlns="69774094-9380-4fae-b934-13dda1a7dd00">
-      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    </lcf76f155ced4ddcb4097134ff3c332f>
-  </documentManagement>
-</p:properties>
+<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{1EADD28A-BF2C-45E6-83DF-53D59D707908}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="399697c3-5931-482a-bf60-528e1410a718"/>
+    <ds:schemaRef ds:uri="69774094-9380-4fae-b934-13dda1a7dd00"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
 
-<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{1860C180-34A5-4519-8E01-EE45D69AD4EA}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
@@ -1033,23 +1082,4 @@
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/internal/obd"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{065CC945-652E-4DFC-A1A9-9FF2FC932111}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{1EADD28A-BF2C-45E6-83DF-53D59D707908}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <ds:schemaRef ds:uri="399697c3-5931-482a-bf60-528e1410a718"/>
-    <ds:schemaRef ds:uri="69774094-9380-4fae-b934-13dda1a7dd00"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
 </file>
</xml_diff>

<commit_message>
Updated downloading client config from google drive
</commit_message>
<xml_diff>
--- a/Config/Client_Config.xlsx
+++ b/Config/Client_Config.xlsx
@@ -779,12 +779,14 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement>
+    <TaxCatchAll xmlns="399697c3-5931-482a-bf60-528e1410a718" xsi:nil="true"/>
+    <lcf76f155ced4ddcb4097134ff3c332f xmlns="69774094-9380-4fae-b934-13dda1a7dd00">
+      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    </lcf76f155ced4ddcb4097134ff3c332f>
+  </documentManagement>
+</p:properties>
 </file>
 
 <file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
@@ -1043,20 +1045,21 @@
 </file>
 
 <file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement>
-    <TaxCatchAll xmlns="399697c3-5931-482a-bf60-528e1410a718" xsi:nil="true"/>
-    <lcf76f155ced4ddcb4097134ff3c332f xmlns="69774094-9380-4fae-b934-13dda1a7dd00">
-      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    </lcf76f155ced4ddcb4097134ff3c332f>
-  </documentManagement>
-</p:properties>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
 </file>
 
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{065CC945-652E-4DFC-A1A9-9FF2FC932111}">
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{1EADD28A-BF2C-45E6-83DF-53D59D707908}">
   <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="399697c3-5931-482a-bf60-528e1410a718"/>
+    <ds:schemaRef ds:uri="69774094-9380-4fae-b934-13dda1a7dd00"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
 </file>
@@ -1081,12 +1084,9 @@
 </file>
 
 <file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{1EADD28A-BF2C-45E6-83DF-53D59D707908}">
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{065CC945-652E-4DFC-A1A9-9FF2FC932111}">
   <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <ds:schemaRef ds:uri="399697c3-5931-482a-bf60-528e1410a718"/>
-    <ds:schemaRef ds:uri="69774094-9380-4fae-b934-13dda1a7dd00"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
 </file>
</xml_diff>